<commit_message>
lean on limpa and limma for every step and preview the intensities before trusting them
</commit_message>
<xml_diff>
--- a/01_Processing/01_Precursors/c_data/precursors.xlsx
+++ b/01_Processing/01_Precursors/c_data/precursors.xlsx
@@ -10,18 +10,17 @@
     <sheet name="read_me" sheetId="1" r:id="rId1"/>
     <sheet name="columns" sheetId="2" r:id="rId2"/>
     <sheet name="run_map" sheetId="3" r:id="rId3"/>
-    <sheet name="q_filters" sheetId="4" r:id="rId4"/>
-    <sheet name="filter_log" sheetId="5" r:id="rId5"/>
-    <sheet name="per_run" sheetId="6" r:id="rId6"/>
-    <sheet name="input_manifest" sheetId="7" r:id="rId7"/>
-    <sheet name="package_versions" sheetId="8" r:id="rId8"/>
+    <sheet name="filter_log" sheetId="4" r:id="rId4"/>
+    <sheet name="per_run" sheetId="5" r:id="rId5"/>
+    <sheet name="input_manifest" sheetId="6" r:id="rId6"/>
+    <sheet name="package_versions" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="314">
   <si>
     <t>sheet</t>
   </si>
@@ -41,16 +40,10 @@
     <t>Every run in the report: biopsy, injection, precursors detected, and whether it was kept.</t>
   </si>
   <si>
-    <t>q_filters</t>
-  </si>
-  <si>
-    <t>Distinct precursors passing the MBR q-values (used) and the no-MBR q-values.</t>
-  </si>
-  <si>
     <t>filter_log</t>
   </si>
   <si>
-    <t>Precursors and proteins after each step.</t>
+    <t>Precursors and proteins before and after the identity filters.</t>
   </si>
   <si>
     <t>per_run</t>
@@ -113,442 +106,421 @@
     <t>Whether this run is the biopsy's kept injection (most precursors among its injections).</t>
   </si>
   <si>
-    <t>filter</t>
-  </si>
-  <si>
-    <t>q-value columns used to keep a precursor.</t>
-  </si>
-  <si>
-    <t>distinct_precursors</t>
-  </si>
-  <si>
-    <t>Distinct precursors passing the q-value filter in at least one run.</t>
-  </si>
-  <si>
-    <t>step</t>
-  </si>
-  <si>
-    <t>Filtering step.</t>
+    <t>count</t>
+  </si>
+  <si>
+    <t>What is counted: precursors or protein groups.</t>
+  </si>
+  <si>
+    <t>before</t>
+  </si>
+  <si>
+    <t>Count before the identity filters.</t>
+  </si>
+  <si>
+    <t>after</t>
+  </si>
+  <si>
+    <t>Count after the identity filters.</t>
+  </si>
+  <si>
+    <t>n_proteins</t>
+  </si>
+  <si>
+    <t>Protein groups with at least one precursor detected in the run.</t>
+  </si>
+  <si>
+    <t>group</t>
+  </si>
+  <si>
+    <t>Group the row belongs to: HR or LR, or C1 or C2 in a proteome grouping.</t>
+  </si>
+  <si>
+    <t>timepoint</t>
+  </si>
+  <si>
+    <t>T1 baseline, T2 after training, T3 after the acute bout at the end of training.</t>
+  </si>
+  <si>
+    <t>input</t>
+  </si>
+  <si>
+    <t>Name the script gives the file it read.</t>
+  </si>
+  <si>
+    <t>path</t>
+  </si>
+  <si>
+    <t>Path of the file read.</t>
+  </si>
+  <si>
+    <t>md5</t>
+  </si>
+  <si>
+    <t>MD5 checksum of the file read.</t>
+  </si>
+  <si>
+    <t>package</t>
+  </si>
+  <si>
+    <t>R package.</t>
+  </si>
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>Package version.</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>Where the package came from.</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S03-T1</t>
+  </si>
+  <si>
+    <t>S03_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S03-T2</t>
+  </si>
+  <si>
+    <t>S03_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S03-T3</t>
+  </si>
+  <si>
+    <t>S03_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S04-T1r</t>
+  </si>
+  <si>
+    <t>S04_T1</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S04-T2</t>
+  </si>
+  <si>
+    <t>S04_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S04-T3</t>
+  </si>
+  <si>
+    <t>S04_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S05-T1</t>
+  </si>
+  <si>
+    <t>S05_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S05-T2</t>
+  </si>
+  <si>
+    <t>S05_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S05-T3</t>
+  </si>
+  <si>
+    <t>S05_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S06-T1</t>
+  </si>
+  <si>
+    <t>S06_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S06-T2</t>
+  </si>
+  <si>
+    <t>S06_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S06-T3</t>
+  </si>
+  <si>
+    <t>S06_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S07-T1_4</t>
+  </si>
+  <si>
+    <t>S07_T1</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S07-T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S07-T2</t>
+  </si>
+  <si>
+    <t>S07_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S10-T1</t>
+  </si>
+  <si>
+    <t>S10_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S10-T2r</t>
+  </si>
+  <si>
+    <t>S10_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S10-T3</t>
+  </si>
+  <si>
+    <t>S10_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S12-T1</t>
+  </si>
+  <si>
+    <t>S12_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S12-T2</t>
+  </si>
+  <si>
+    <t>S12_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S12-T3</t>
+  </si>
+  <si>
+    <t>S12_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S13-T1_4</t>
+  </si>
+  <si>
+    <t>S13_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S13-T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S13-T2r</t>
+  </si>
+  <si>
+    <t>S13_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S13-T3</t>
+  </si>
+  <si>
+    <t>S13_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S14-T1r</t>
+  </si>
+  <si>
+    <t>S14_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S14-T2</t>
+  </si>
+  <si>
+    <t>S14_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S14-T3</t>
+  </si>
+  <si>
+    <t>S14_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S16-T1</t>
+  </si>
+  <si>
+    <t>S16_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S16-T2</t>
+  </si>
+  <si>
+    <t>S16_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S16-T3</t>
+  </si>
+  <si>
+    <t>S16_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S17-T1_4</t>
+  </si>
+  <si>
+    <t>S17_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S17-T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S17-T2</t>
+  </si>
+  <si>
+    <t>S17_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S17-T3</t>
+  </si>
+  <si>
+    <t>S17_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S21-T1</t>
+  </si>
+  <si>
+    <t>S21_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S21-T2</t>
+  </si>
+  <si>
+    <t>S21_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S21-T3</t>
+  </si>
+  <si>
+    <t>S21_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S22-T1</t>
+  </si>
+  <si>
+    <t>S22_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S22-T2</t>
+  </si>
+  <si>
+    <t>S22_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S22-T3</t>
+  </si>
+  <si>
+    <t>S22_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S24-T1</t>
+  </si>
+  <si>
+    <t>S24_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S24-T2</t>
+  </si>
+  <si>
+    <t>S24_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S24-T3</t>
+  </si>
+  <si>
+    <t>S24_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S27-T1rr</t>
+  </si>
+  <si>
+    <t>S27_T1</t>
+  </si>
+  <si>
+    <t>rr</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S27-T2</t>
+  </si>
+  <si>
+    <t>S27_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S27-T3r</t>
+  </si>
+  <si>
+    <t>S27_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S28-T1</t>
+  </si>
+  <si>
+    <t>S28_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S28-T2</t>
+  </si>
+  <si>
+    <t>S28_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S28-T3</t>
+  </si>
+  <si>
+    <t>S28_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S29-T1_4</t>
+  </si>
+  <si>
+    <t>S29_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S29-T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S29-T2</t>
+  </si>
+  <si>
+    <t>S29_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S29-T3_r</t>
+  </si>
+  <si>
+    <t>S29_T3</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S30-T1</t>
+  </si>
+  <si>
+    <t>S30_T1</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S30-T2</t>
+  </si>
+  <si>
+    <t>S30_T2</t>
+  </si>
+  <si>
+    <t>JBBC_CL_S30-T3</t>
+  </si>
+  <si>
+    <t>S30_T3</t>
   </si>
   <si>
     <t>precursors</t>
   </si>
   <si>
-    <t>Precursors left after the step.</t>
-  </si>
-  <si>
     <t>proteins</t>
-  </si>
-  <si>
-    <t>Protein groups left after the step.</t>
-  </si>
-  <si>
-    <t>n_proteins</t>
-  </si>
-  <si>
-    <t>Protein groups with at least one precursor detected in the run.</t>
-  </si>
-  <si>
-    <t>group</t>
-  </si>
-  <si>
-    <t>Group the row belongs to: HR or LR, or C1 or C2 in a proteome grouping.</t>
-  </si>
-  <si>
-    <t>timepoint</t>
-  </si>
-  <si>
-    <t>T1 baseline, T2 after training, T3 after the acute bout at the end of training.</t>
-  </si>
-  <si>
-    <t>input</t>
-  </si>
-  <si>
-    <t>Name the script gives the file it read.</t>
-  </si>
-  <si>
-    <t>path</t>
-  </si>
-  <si>
-    <t>Path of the file read.</t>
-  </si>
-  <si>
-    <t>md5</t>
-  </si>
-  <si>
-    <t>MD5 checksum of the file read.</t>
-  </si>
-  <si>
-    <t>package</t>
-  </si>
-  <si>
-    <t>R package.</t>
-  </si>
-  <si>
-    <t>version</t>
-  </si>
-  <si>
-    <t>Package version.</t>
-  </si>
-  <si>
-    <t>source</t>
-  </si>
-  <si>
-    <t>Where the package came from.</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S03-T1</t>
-  </si>
-  <si>
-    <t>S03_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S03-T2</t>
-  </si>
-  <si>
-    <t>S03_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S03-T3</t>
-  </si>
-  <si>
-    <t>S03_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S04-T1r</t>
-  </si>
-  <si>
-    <t>S04_T1</t>
-  </si>
-  <si>
-    <t>r</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S04-T2</t>
-  </si>
-  <si>
-    <t>S04_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S04-T3</t>
-  </si>
-  <si>
-    <t>S04_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S05-T1</t>
-  </si>
-  <si>
-    <t>S05_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S05-T2</t>
-  </si>
-  <si>
-    <t>S05_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S05-T3</t>
-  </si>
-  <si>
-    <t>S05_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S06-T1</t>
-  </si>
-  <si>
-    <t>S06_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S06-T2</t>
-  </si>
-  <si>
-    <t>S06_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S06-T3</t>
-  </si>
-  <si>
-    <t>S06_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S07-T1_4</t>
-  </si>
-  <si>
-    <t>S07_T1</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S07-T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S07-T2</t>
-  </si>
-  <si>
-    <t>S07_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S10-T1</t>
-  </si>
-  <si>
-    <t>S10_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S10-T2r</t>
-  </si>
-  <si>
-    <t>S10_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S10-T3</t>
-  </si>
-  <si>
-    <t>S10_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S12-T1</t>
-  </si>
-  <si>
-    <t>S12_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S12-T2</t>
-  </si>
-  <si>
-    <t>S12_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S12-T3</t>
-  </si>
-  <si>
-    <t>S12_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S13-T1_4</t>
-  </si>
-  <si>
-    <t>S13_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S13-T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S13-T2r</t>
-  </si>
-  <si>
-    <t>S13_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S13-T3</t>
-  </si>
-  <si>
-    <t>S13_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S14-T1r</t>
-  </si>
-  <si>
-    <t>S14_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S14-T2</t>
-  </si>
-  <si>
-    <t>S14_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S14-T3</t>
-  </si>
-  <si>
-    <t>S14_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S16-T1</t>
-  </si>
-  <si>
-    <t>S16_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S16-T2</t>
-  </si>
-  <si>
-    <t>S16_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S16-T3</t>
-  </si>
-  <si>
-    <t>S16_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S17-T1_4</t>
-  </si>
-  <si>
-    <t>S17_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S17-T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S17-T2</t>
-  </si>
-  <si>
-    <t>S17_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S17-T3</t>
-  </si>
-  <si>
-    <t>S17_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S21-T1</t>
-  </si>
-  <si>
-    <t>S21_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S21-T2</t>
-  </si>
-  <si>
-    <t>S21_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S21-T3</t>
-  </si>
-  <si>
-    <t>S21_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S22-T1</t>
-  </si>
-  <si>
-    <t>S22_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S22-T2</t>
-  </si>
-  <si>
-    <t>S22_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S22-T3</t>
-  </si>
-  <si>
-    <t>S22_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S24-T1</t>
-  </si>
-  <si>
-    <t>S24_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S24-T2</t>
-  </si>
-  <si>
-    <t>S24_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S24-T3</t>
-  </si>
-  <si>
-    <t>S24_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S27-T1rr</t>
-  </si>
-  <si>
-    <t>S27_T1</t>
-  </si>
-  <si>
-    <t>rr</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S27-T2</t>
-  </si>
-  <si>
-    <t>S27_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S27-T3r</t>
-  </si>
-  <si>
-    <t>S27_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S28-T1</t>
-  </si>
-  <si>
-    <t>S28_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S28-T2</t>
-  </si>
-  <si>
-    <t>S28_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S28-T3</t>
-  </si>
-  <si>
-    <t>S28_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S29-T1_4</t>
-  </si>
-  <si>
-    <t>S29_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S29-T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S29-T2</t>
-  </si>
-  <si>
-    <t>S29_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S29-T3_r</t>
-  </si>
-  <si>
-    <t>S29_T3</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S30-T1</t>
-  </si>
-  <si>
-    <t>S30_T1</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S30-T2</t>
-  </si>
-  <si>
-    <t>S30_T2</t>
-  </si>
-  <si>
-    <t>JBBC_CL_S30-T3</t>
-  </si>
-  <si>
-    <t>S30_T3</t>
-  </si>
-  <si>
-    <t>MBR (used)</t>
-  </si>
-  <si>
-    <t>no MBR</t>
-  </si>
-  <si>
-    <t>chosen runs</t>
-  </si>
-  <si>
-    <t>proteotypic precursors only</t>
-  </si>
-  <si>
-    <t>single-protein groups only</t>
   </si>
   <si>
     <t>HR</t>
@@ -1332,7 +1304,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1">
@@ -1389,14 +1361,6 @@
       </c>
       <c r="B7" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1406,7 +1370,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1414,10 +1378,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1425,10 +1389,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1436,10 +1400,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1447,10 +1411,10 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1458,10 +1422,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1469,10 +1433,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1480,10 +1444,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1491,10 +1455,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1502,21 +1466,21 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1524,10 +1488,10 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1535,43 +1499,43 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1579,10 +1543,10 @@
         <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1590,21 +1554,21 @@
         <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C18" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1612,10 +1576,10 @@
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C19" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1623,43 +1587,21 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" t="s">
-        <v>14</v>
-      </c>
-      <c r="B22" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" t="s">
-        <v>14</v>
-      </c>
-      <c r="B23" t="s">
-        <v>56</v>
-      </c>
-      <c r="C23" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1674,33 +1616,33 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B2">
         <v>10875</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -1711,13 +1653,13 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B3">
         <v>13066</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
@@ -1728,13 +1670,13 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B4">
         <v>14861</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -1745,16 +1687,16 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B5">
         <v>14665</v>
       </c>
       <c r="C5" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -1765,13 +1707,13 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>16656</v>
       </c>
       <c r="C6" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -1782,13 +1724,13 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B7">
         <v>13762</v>
       </c>
       <c r="C7" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
@@ -1799,13 +1741,13 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B8">
         <v>15037</v>
       </c>
       <c r="C8" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
@@ -1816,13 +1758,13 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B9">
         <v>15641</v>
       </c>
       <c r="C9" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
@@ -1833,13 +1775,13 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B10">
         <v>11783</v>
       </c>
       <c r="C10" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -1850,13 +1792,13 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B11">
         <v>10204</v>
       </c>
       <c r="C11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="E11" t="b">
         <v>1</v>
@@ -1867,13 +1809,13 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B12">
         <v>14920</v>
       </c>
       <c r="C12" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E12" t="b">
         <v>1</v>
@@ -1884,13 +1826,13 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B13">
         <v>14715</v>
       </c>
       <c r="C13" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E13" t="b">
         <v>1</v>
@@ -1901,16 +1843,16 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B14">
         <v>14576</v>
       </c>
       <c r="C14" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -1921,13 +1863,13 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B15">
         <v>11819</v>
       </c>
       <c r="C15" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -1938,13 +1880,13 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B16">
         <v>11296</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -1955,13 +1897,13 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B17">
         <v>13041</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E17" t="b">
         <v>1</v>
@@ -1972,16 +1914,16 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B18">
         <v>8305</v>
       </c>
       <c r="C18" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D18" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E18" t="b">
         <v>1</v>
@@ -1992,13 +1934,13 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B19">
         <v>12044</v>
       </c>
       <c r="C19" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E19" t="b">
         <v>1</v>
@@ -2009,13 +1951,13 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B20">
         <v>14142</v>
       </c>
       <c r="C20" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E20" t="b">
         <v>1</v>
@@ -2026,13 +1968,13 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B21">
         <v>13814</v>
       </c>
       <c r="C21" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E21" t="b">
         <v>1</v>
@@ -2043,13 +1985,13 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B22">
         <v>13038</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E22" t="b">
         <v>1</v>
@@ -2060,16 +2002,16 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B23">
         <v>361</v>
       </c>
       <c r="C23" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D23" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -2080,13 +2022,13 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B24">
         <v>255</v>
       </c>
       <c r="C24" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -2097,16 +2039,16 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B25">
         <v>10578</v>
       </c>
       <c r="C25" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="D25" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -2117,13 +2059,13 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="B26">
         <v>9696</v>
       </c>
       <c r="C26" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -2134,16 +2076,16 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B27">
         <v>13461</v>
       </c>
       <c r="C27" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D27" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E27" t="b">
         <v>1</v>
@@ -2154,13 +2096,13 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B28">
         <v>13299</v>
       </c>
       <c r="C28" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E28" t="b">
         <v>1</v>
@@ -2171,13 +2113,13 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B29">
         <v>14763</v>
       </c>
       <c r="C29" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="E29" t="b">
         <v>1</v>
@@ -2188,13 +2130,13 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B30">
         <v>11178</v>
       </c>
       <c r="C30" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E30" t="b">
         <v>1</v>
@@ -2205,13 +2147,13 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B31">
         <v>14444</v>
       </c>
       <c r="C31" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="E31" t="b">
         <v>1</v>
@@ -2222,13 +2164,13 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B32">
         <v>14559</v>
       </c>
       <c r="C32" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E32" t="b">
         <v>1</v>
@@ -2239,16 +2181,16 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B33">
         <v>10886</v>
       </c>
       <c r="C33" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D33" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E33" t="b">
         <v>1</v>
@@ -2259,13 +2201,13 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="B34">
         <v>10162</v>
       </c>
       <c r="C34" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="E34" t="b">
         <v>1</v>
@@ -2276,13 +2218,13 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B35">
         <v>11456</v>
       </c>
       <c r="C35" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E35" t="b">
         <v>1</v>
@@ -2293,13 +2235,13 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B36">
         <v>14305</v>
       </c>
       <c r="C36" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E36" t="b">
         <v>1</v>
@@ -2310,13 +2252,13 @@
     </row>
     <row r="37" spans="1:6">
       <c r="A37" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B37">
         <v>13069</v>
       </c>
       <c r="C37" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="E37" t="b">
         <v>1</v>
@@ -2327,13 +2269,13 @@
     </row>
     <row r="38" spans="1:6">
       <c r="A38" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B38">
         <v>13638</v>
       </c>
       <c r="C38" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E38" t="b">
         <v>1</v>
@@ -2344,13 +2286,13 @@
     </row>
     <row r="39" spans="1:6">
       <c r="A39" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="B39">
         <v>12024</v>
       </c>
       <c r="C39" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="E39" t="b">
         <v>1</v>
@@ -2361,13 +2303,13 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="B40">
         <v>11947</v>
       </c>
       <c r="C40" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="E40" t="b">
         <v>1</v>
@@ -2378,13 +2320,13 @@
     </row>
     <row r="41" spans="1:6">
       <c r="A41" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B41">
         <v>14888</v>
       </c>
       <c r="C41" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="E41" t="b">
         <v>1</v>
@@ -2395,13 +2337,13 @@
     </row>
     <row r="42" spans="1:6">
       <c r="A42" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="B42">
         <v>13631</v>
       </c>
       <c r="C42" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="E42" t="b">
         <v>1</v>
@@ -2412,13 +2354,13 @@
     </row>
     <row r="43" spans="1:6">
       <c r="A43" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="B43">
         <v>12310</v>
       </c>
       <c r="C43" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E43" t="b">
         <v>1</v>
@@ -2429,13 +2371,13 @@
     </row>
     <row r="44" spans="1:6">
       <c r="A44" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="B44">
         <v>12668</v>
       </c>
       <c r="C44" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E44" t="b">
         <v>1</v>
@@ -2446,13 +2388,13 @@
     </row>
     <row r="45" spans="1:6">
       <c r="A45" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="B45">
         <v>13026</v>
       </c>
       <c r="C45" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="E45" t="b">
         <v>1</v>
@@ -2463,16 +2405,16 @@
     </row>
     <row r="46" spans="1:6">
       <c r="A46" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="B46">
         <v>12825</v>
       </c>
       <c r="C46" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="D46" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="E46" t="b">
         <v>1</v>
@@ -2483,13 +2425,13 @@
     </row>
     <row r="47" spans="1:6">
       <c r="A47" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="B47">
         <v>15415</v>
       </c>
       <c r="C47" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="E47" t="b">
         <v>1</v>
@@ -2500,16 +2442,16 @@
     </row>
     <row r="48" spans="1:6">
       <c r="A48" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B48">
         <v>12545</v>
       </c>
       <c r="C48" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="D48" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E48" t="b">
         <v>1</v>
@@ -2520,13 +2462,13 @@
     </row>
     <row r="49" spans="1:6">
       <c r="A49" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="B49">
         <v>15218</v>
       </c>
       <c r="C49" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="E49" t="b">
         <v>1</v>
@@ -2537,13 +2479,13 @@
     </row>
     <row r="50" spans="1:6">
       <c r="A50" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="B50">
         <v>6699</v>
       </c>
       <c r="C50" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E50" t="b">
         <v>1</v>
@@ -2554,13 +2496,13 @@
     </row>
     <row r="51" spans="1:6">
       <c r="A51" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B51">
         <v>4048</v>
       </c>
       <c r="C51" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="E51" t="b">
         <v>1</v>
@@ -2571,16 +2513,16 @@
     </row>
     <row r="52" spans="1:6">
       <c r="A52" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="B52">
         <v>12605</v>
       </c>
       <c r="C52" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D52" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E52" t="b">
         <v>1</v>
@@ -2591,13 +2533,13 @@
     </row>
     <row r="53" spans="1:6">
       <c r="A53" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B53">
         <v>8551</v>
       </c>
       <c r="C53" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="E53" t="b">
         <v>1</v>
@@ -2608,13 +2550,13 @@
     </row>
     <row r="54" spans="1:6">
       <c r="A54" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B54">
         <v>13135</v>
       </c>
       <c r="C54" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="E54" t="b">
         <v>1</v>
@@ -2625,16 +2567,16 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B55">
         <v>12856</v>
       </c>
       <c r="C55" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="D55" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E55" t="b">
         <v>1</v>
@@ -2645,13 +2587,13 @@
     </row>
     <row r="56" spans="1:6">
       <c r="A56" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="B56">
         <v>13407</v>
       </c>
       <c r="C56" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="E56" t="b">
         <v>1</v>
@@ -2662,13 +2604,13 @@
     </row>
     <row r="57" spans="1:6">
       <c r="A57" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B57">
         <v>14802</v>
       </c>
       <c r="C57" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="E57" t="b">
         <v>1</v>
@@ -2679,13 +2621,13 @@
     </row>
     <row r="58" spans="1:6">
       <c r="A58" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="B58">
         <v>11992</v>
       </c>
       <c r="C58" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="E58" t="b">
         <v>1</v>
@@ -2701,31 +2643,40 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1">
+    <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B2">
-        <v>22389</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>22342</v>
+      </c>
+      <c r="C2">
+        <v>22342</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="B3">
-        <v>19936</v>
+        <v>2401</v>
+      </c>
+      <c r="C3">
+        <v>2401</v>
       </c>
     </row>
   </sheetData>
@@ -2735,51 +2686,840 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1">
+    <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
       <c r="B2">
-        <v>22342</v>
+        <v>4048</v>
       </c>
       <c r="C2">
-        <v>2401</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>810</v>
+      </c>
+      <c r="D2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>174</v>
+        <v>149</v>
       </c>
       <c r="B3">
-        <v>22342</v>
+        <v>6699</v>
       </c>
       <c r="C3">
-        <v>2401</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+        <v>1061</v>
+      </c>
+      <c r="D3" t="s">
+        <v>167</v>
+      </c>
+      <c r="E3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>175</v>
+        <v>86</v>
       </c>
       <c r="B4">
-        <v>22342</v>
+        <v>8305</v>
       </c>
       <c r="C4">
-        <v>2401</v>
+        <v>1490</v>
+      </c>
+      <c r="D4" t="s">
+        <v>167</v>
+      </c>
+      <c r="E4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5">
+        <v>10204</v>
+      </c>
+      <c r="C5">
+        <v>1597</v>
+      </c>
+      <c r="D5" t="s">
+        <v>170</v>
+      </c>
+      <c r="E5" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6">
+        <v>10875</v>
+      </c>
+      <c r="C6">
+        <v>1521</v>
+      </c>
+      <c r="D6" t="s">
+        <v>167</v>
+      </c>
+      <c r="E6" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B7">
+        <v>10886</v>
+      </c>
+      <c r="C7">
+        <v>1717</v>
+      </c>
+      <c r="D7" t="s">
+        <v>170</v>
+      </c>
+      <c r="E7" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B8">
+        <v>11178</v>
+      </c>
+      <c r="C8">
+        <v>1745</v>
+      </c>
+      <c r="D8" t="s">
+        <v>167</v>
+      </c>
+      <c r="E8" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B9">
+        <v>11456</v>
+      </c>
+      <c r="C9">
+        <v>1688</v>
+      </c>
+      <c r="D9" t="s">
+        <v>170</v>
+      </c>
+      <c r="E9" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10">
+        <v>11783</v>
+      </c>
+      <c r="C10">
+        <v>1738</v>
+      </c>
+      <c r="D10" t="s">
+        <v>170</v>
+      </c>
+      <c r="E10" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>128</v>
+      </c>
+      <c r="B11">
+        <v>11947</v>
+      </c>
+      <c r="C11">
+        <v>1869</v>
+      </c>
+      <c r="D11" t="s">
+        <v>167</v>
+      </c>
+      <c r="E11" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>164</v>
+      </c>
+      <c r="B12">
+        <v>11992</v>
+      </c>
+      <c r="C12">
+        <v>1911</v>
+      </c>
+      <c r="D12" t="s">
+        <v>170</v>
+      </c>
+      <c r="E12" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>126</v>
+      </c>
+      <c r="B13">
+        <v>12024</v>
+      </c>
+      <c r="C13">
+        <v>1728</v>
+      </c>
+      <c r="D13" t="s">
+        <v>170</v>
+      </c>
+      <c r="E13" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14">
+        <v>12044</v>
+      </c>
+      <c r="C14">
+        <v>1853</v>
+      </c>
+      <c r="D14" t="s">
+        <v>167</v>
+      </c>
+      <c r="E14" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>134</v>
+      </c>
+      <c r="B15">
+        <v>12310</v>
+      </c>
+      <c r="C15">
+        <v>1840</v>
+      </c>
+      <c r="D15" t="s">
+        <v>167</v>
+      </c>
+      <c r="E15" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>145</v>
+      </c>
+      <c r="B16">
+        <v>12545</v>
+      </c>
+      <c r="C16">
+        <v>1806</v>
+      </c>
+      <c r="D16" t="s">
+        <v>167</v>
+      </c>
+      <c r="E16" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>153</v>
+      </c>
+      <c r="B17">
+        <v>12605</v>
+      </c>
+      <c r="C17">
+        <v>1810</v>
+      </c>
+      <c r="D17" t="s">
+        <v>167</v>
+      </c>
+      <c r="E17" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18">
+        <v>12668</v>
+      </c>
+      <c r="C18">
+        <v>1815</v>
+      </c>
+      <c r="D18" t="s">
+        <v>167</v>
+      </c>
+      <c r="E18" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>140</v>
+      </c>
+      <c r="B19">
+        <v>12825</v>
+      </c>
+      <c r="C19">
+        <v>1859</v>
+      </c>
+      <c r="D19" t="s">
+        <v>167</v>
+      </c>
+      <c r="E19" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>158</v>
+      </c>
+      <c r="B20">
+        <v>12856</v>
+      </c>
+      <c r="C20">
+        <v>1793</v>
+      </c>
+      <c r="D20" t="s">
+        <v>167</v>
+      </c>
+      <c r="E20" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>138</v>
+      </c>
+      <c r="B21">
+        <v>13026</v>
+      </c>
+      <c r="C21">
+        <v>1951</v>
+      </c>
+      <c r="D21" t="s">
+        <v>167</v>
+      </c>
+      <c r="E21" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>94</v>
+      </c>
+      <c r="B22">
+        <v>13038</v>
+      </c>
+      <c r="C22">
+        <v>1833</v>
+      </c>
+      <c r="D22" t="s">
+        <v>170</v>
+      </c>
+      <c r="E22" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23">
+        <v>13041</v>
+      </c>
+      <c r="C23">
+        <v>1768</v>
+      </c>
+      <c r="D23" t="s">
+        <v>167</v>
+      </c>
+      <c r="E23" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24">
+        <v>13066</v>
+      </c>
+      <c r="C24">
+        <v>1884</v>
+      </c>
+      <c r="D24" t="s">
+        <v>167</v>
+      </c>
+      <c r="E24" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>122</v>
+      </c>
+      <c r="B25">
+        <v>13069</v>
+      </c>
+      <c r="C25">
+        <v>1846</v>
+      </c>
+      <c r="D25" t="s">
+        <v>170</v>
+      </c>
+      <c r="E25" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>156</v>
+      </c>
+      <c r="B26">
+        <v>13135</v>
+      </c>
+      <c r="C26">
+        <v>1977</v>
+      </c>
+      <c r="D26" t="s">
+        <v>167</v>
+      </c>
+      <c r="E26" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" t="s">
+        <v>105</v>
+      </c>
+      <c r="B27">
+        <v>13299</v>
+      </c>
+      <c r="C27">
+        <v>1982</v>
+      </c>
+      <c r="D27" t="s">
+        <v>170</v>
+      </c>
+      <c r="E27" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" t="s">
+        <v>160</v>
+      </c>
+      <c r="B28">
+        <v>13407</v>
+      </c>
+      <c r="C28">
+        <v>1994</v>
+      </c>
+      <c r="D28" t="s">
+        <v>170</v>
+      </c>
+      <c r="E28" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" t="s">
+        <v>103</v>
+      </c>
+      <c r="B29">
+        <v>13461</v>
+      </c>
+      <c r="C29">
+        <v>1926</v>
+      </c>
+      <c r="D29" t="s">
+        <v>170</v>
+      </c>
+      <c r="E29" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" t="s">
+        <v>132</v>
+      </c>
+      <c r="B30">
+        <v>13631</v>
+      </c>
+      <c r="C30">
+        <v>2001</v>
+      </c>
+      <c r="D30" t="s">
+        <v>167</v>
+      </c>
+      <c r="E30" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" t="s">
+        <v>124</v>
+      </c>
+      <c r="B31">
+        <v>13638</v>
+      </c>
+      <c r="C31">
+        <v>1963</v>
+      </c>
+      <c r="D31" t="s">
+        <v>170</v>
+      </c>
+      <c r="E31" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32">
+        <v>13762</v>
+      </c>
+      <c r="C32">
+        <v>1962</v>
+      </c>
+      <c r="D32" t="s">
+        <v>170</v>
+      </c>
+      <c r="E32" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" t="s">
+        <v>92</v>
+      </c>
+      <c r="B33">
+        <v>13814</v>
+      </c>
+      <c r="C33">
+        <v>1928</v>
+      </c>
+      <c r="D33" t="s">
+        <v>170</v>
+      </c>
+      <c r="E33" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" t="s">
+        <v>90</v>
+      </c>
+      <c r="B34">
+        <v>14142</v>
+      </c>
+      <c r="C34">
+        <v>1912</v>
+      </c>
+      <c r="D34" t="s">
+        <v>170</v>
+      </c>
+      <c r="E34" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" t="s">
+        <v>120</v>
+      </c>
+      <c r="B35">
+        <v>14305</v>
+      </c>
+      <c r="C35">
+        <v>2047</v>
+      </c>
+      <c r="D35" t="s">
+        <v>170</v>
+      </c>
+      <c r="E35" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" t="s">
+        <v>111</v>
+      </c>
+      <c r="B36">
+        <v>14444</v>
+      </c>
+      <c r="C36">
+        <v>2015</v>
+      </c>
+      <c r="D36" t="s">
+        <v>167</v>
+      </c>
+      <c r="E36" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" t="s">
+        <v>113</v>
+      </c>
+      <c r="B37">
+        <v>14559</v>
+      </c>
+      <c r="C37">
+        <v>1994</v>
+      </c>
+      <c r="D37" t="s">
+        <v>167</v>
+      </c>
+      <c r="E37" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>14665</v>
+      </c>
+      <c r="C38">
+        <v>2039</v>
+      </c>
+      <c r="D38" t="s">
+        <v>170</v>
+      </c>
+      <c r="E38" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" t="s">
+        <v>76</v>
+      </c>
+      <c r="B39">
+        <v>14715</v>
+      </c>
+      <c r="C39">
+        <v>2002</v>
+      </c>
+      <c r="D39" t="s">
+        <v>170</v>
+      </c>
+      <c r="E39" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" t="s">
+        <v>107</v>
+      </c>
+      <c r="B40">
+        <v>14763</v>
+      </c>
+      <c r="C40">
+        <v>2028</v>
+      </c>
+      <c r="D40" t="s">
+        <v>170</v>
+      </c>
+      <c r="E40" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" t="s">
+        <v>162</v>
+      </c>
+      <c r="B41">
+        <v>14802</v>
+      </c>
+      <c r="C41">
+        <v>2038</v>
+      </c>
+      <c r="D41" t="s">
+        <v>170</v>
+      </c>
+      <c r="E41" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" t="s">
+        <v>57</v>
+      </c>
+      <c r="B42">
+        <v>14861</v>
+      </c>
+      <c r="C42">
+        <v>2069</v>
+      </c>
+      <c r="D42" t="s">
+        <v>167</v>
+      </c>
+      <c r="E42" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" t="s">
+        <v>130</v>
+      </c>
+      <c r="B43">
+        <v>14888</v>
+      </c>
+      <c r="C43">
+        <v>2080</v>
+      </c>
+      <c r="D43" t="s">
+        <v>167</v>
+      </c>
+      <c r="E43" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44">
+        <v>14920</v>
+      </c>
+      <c r="C44">
+        <v>2070</v>
+      </c>
+      <c r="D44" t="s">
+        <v>170</v>
+      </c>
+      <c r="E44" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" t="s">
+        <v>66</v>
+      </c>
+      <c r="B45">
+        <v>15037</v>
+      </c>
+      <c r="C45">
+        <v>1966</v>
+      </c>
+      <c r="D45" t="s">
+        <v>170</v>
+      </c>
+      <c r="E45" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" t="s">
+        <v>147</v>
+      </c>
+      <c r="B46">
+        <v>15218</v>
+      </c>
+      <c r="C46">
+        <v>1954</v>
+      </c>
+      <c r="D46" t="s">
+        <v>167</v>
+      </c>
+      <c r="E46" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" t="s">
+        <v>143</v>
+      </c>
+      <c r="B47">
+        <v>15415</v>
+      </c>
+      <c r="C47">
+        <v>2061</v>
+      </c>
+      <c r="D47" t="s">
+        <v>167</v>
+      </c>
+      <c r="E47" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" t="s">
+        <v>68</v>
+      </c>
+      <c r="B48">
+        <v>15641</v>
+      </c>
+      <c r="C48">
+        <v>2043</v>
+      </c>
+      <c r="D48" t="s">
+        <v>170</v>
+      </c>
+      <c r="E48" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49">
+        <v>16656</v>
+      </c>
+      <c r="C49">
+        <v>2070</v>
+      </c>
+      <c r="D49" t="s">
+        <v>170</v>
+      </c>
+      <c r="E49" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -2789,840 +3529,40 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1">
+    <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>157</v>
-      </c>
-      <c r="B2">
-        <v>4048</v>
-      </c>
-      <c r="C2">
-        <v>810</v>
-      </c>
-      <c r="D2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B3" t="s">
         <v>176</v>
       </c>
-      <c r="E2" t="s">
+      <c r="C3" t="s">
         <v>177</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B3">
-        <v>6699</v>
-      </c>
-      <c r="C3">
-        <v>1061</v>
-      </c>
-      <c r="D3" t="s">
-        <v>176</v>
-      </c>
-      <c r="E3" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>92</v>
-      </c>
-      <c r="B4">
-        <v>8305</v>
-      </c>
-      <c r="C4">
-        <v>1490</v>
-      </c>
-      <c r="D4" t="s">
-        <v>176</v>
-      </c>
-      <c r="E4" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B5">
-        <v>10204</v>
-      </c>
-      <c r="C5">
-        <v>1597</v>
-      </c>
-      <c r="D5" t="s">
-        <v>179</v>
-      </c>
-      <c r="E5" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B6">
-        <v>10875</v>
-      </c>
-      <c r="C6">
-        <v>1521</v>
-      </c>
-      <c r="D6" t="s">
-        <v>176</v>
-      </c>
-      <c r="E6" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>121</v>
-      </c>
-      <c r="B7">
-        <v>10886</v>
-      </c>
-      <c r="C7">
-        <v>1717</v>
-      </c>
-      <c r="D7" t="s">
-        <v>179</v>
-      </c>
-      <c r="E7" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>115</v>
-      </c>
-      <c r="B8">
-        <v>11178</v>
-      </c>
-      <c r="C8">
-        <v>1745</v>
-      </c>
-      <c r="D8" t="s">
-        <v>176</v>
-      </c>
-      <c r="E8" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
-        <v>124</v>
-      </c>
-      <c r="B9">
-        <v>11456</v>
-      </c>
-      <c r="C9">
-        <v>1688</v>
-      </c>
-      <c r="D9" t="s">
-        <v>179</v>
-      </c>
-      <c r="E9" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" t="s">
-        <v>76</v>
-      </c>
-      <c r="B10">
-        <v>11783</v>
-      </c>
-      <c r="C10">
-        <v>1738</v>
-      </c>
-      <c r="D10" t="s">
-        <v>179</v>
-      </c>
-      <c r="E10" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" t="s">
-        <v>134</v>
-      </c>
-      <c r="B11">
-        <v>11947</v>
-      </c>
-      <c r="C11">
-        <v>1869</v>
-      </c>
-      <c r="D11" t="s">
-        <v>176</v>
-      </c>
-      <c r="E11" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
-        <v>170</v>
-      </c>
-      <c r="B12">
-        <v>11992</v>
-      </c>
-      <c r="C12">
-        <v>1911</v>
-      </c>
-      <c r="D12" t="s">
-        <v>179</v>
-      </c>
-      <c r="E12" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" t="s">
-        <v>132</v>
-      </c>
-      <c r="B13">
-        <v>12024</v>
-      </c>
-      <c r="C13">
-        <v>1728</v>
-      </c>
-      <c r="D13" t="s">
-        <v>179</v>
-      </c>
-      <c r="E13" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" t="s">
-        <v>94</v>
-      </c>
-      <c r="B14">
-        <v>12044</v>
-      </c>
-      <c r="C14">
-        <v>1853</v>
-      </c>
-      <c r="D14" t="s">
-        <v>176</v>
-      </c>
-      <c r="E14" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" t="s">
-        <v>140</v>
-      </c>
-      <c r="B15">
-        <v>12310</v>
-      </c>
-      <c r="C15">
-        <v>1840</v>
-      </c>
-      <c r="D15" t="s">
-        <v>176</v>
-      </c>
-      <c r="E15" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" t="s">
-        <v>151</v>
-      </c>
-      <c r="B16">
-        <v>12545</v>
-      </c>
-      <c r="C16">
-        <v>1806</v>
-      </c>
-      <c r="D16" t="s">
-        <v>176</v>
-      </c>
-      <c r="E16" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" t="s">
-        <v>159</v>
-      </c>
-      <c r="B17">
-        <v>12605</v>
-      </c>
-      <c r="C17">
-        <v>1810</v>
-      </c>
-      <c r="D17" t="s">
-        <v>176</v>
-      </c>
-      <c r="E17" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" t="s">
-        <v>142</v>
-      </c>
-      <c r="B18">
-        <v>12668</v>
-      </c>
-      <c r="C18">
-        <v>1815</v>
-      </c>
-      <c r="D18" t="s">
-        <v>176</v>
-      </c>
-      <c r="E18" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" t="s">
-        <v>146</v>
-      </c>
-      <c r="B19">
-        <v>12825</v>
-      </c>
-      <c r="C19">
-        <v>1859</v>
-      </c>
-      <c r="D19" t="s">
-        <v>176</v>
-      </c>
-      <c r="E19" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" t="s">
-        <v>164</v>
-      </c>
-      <c r="B20">
-        <v>12856</v>
-      </c>
-      <c r="C20">
-        <v>1793</v>
-      </c>
-      <c r="D20" t="s">
-        <v>176</v>
-      </c>
-      <c r="E20" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" t="s">
-        <v>144</v>
-      </c>
-      <c r="B21">
-        <v>13026</v>
-      </c>
-      <c r="C21">
-        <v>1951</v>
-      </c>
-      <c r="D21" t="s">
-        <v>176</v>
-      </c>
-      <c r="E21" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" t="s">
-        <v>100</v>
-      </c>
-      <c r="B22">
-        <v>13038</v>
-      </c>
-      <c r="C22">
-        <v>1833</v>
-      </c>
-      <c r="D22" t="s">
-        <v>179</v>
-      </c>
-      <c r="E22" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" t="s">
-        <v>90</v>
-      </c>
-      <c r="B23">
-        <v>13041</v>
-      </c>
-      <c r="C23">
-        <v>1768</v>
-      </c>
-      <c r="D23" t="s">
-        <v>176</v>
-      </c>
-      <c r="E23" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" t="s">
-        <v>61</v>
-      </c>
-      <c r="B24">
-        <v>13066</v>
-      </c>
-      <c r="C24">
-        <v>1884</v>
-      </c>
-      <c r="D24" t="s">
-        <v>176</v>
-      </c>
-      <c r="E24" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" t="s">
-        <v>128</v>
-      </c>
-      <c r="B25">
-        <v>13069</v>
-      </c>
-      <c r="C25">
-        <v>1846</v>
-      </c>
-      <c r="D25" t="s">
-        <v>179</v>
-      </c>
-      <c r="E25" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" t="s">
-        <v>162</v>
-      </c>
-      <c r="B26">
-        <v>13135</v>
-      </c>
-      <c r="C26">
-        <v>1977</v>
-      </c>
-      <c r="D26" t="s">
-        <v>176</v>
-      </c>
-      <c r="E26" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" t="s">
-        <v>111</v>
-      </c>
-      <c r="B27">
-        <v>13299</v>
-      </c>
-      <c r="C27">
-        <v>1982</v>
-      </c>
-      <c r="D27" t="s">
-        <v>179</v>
-      </c>
-      <c r="E27" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" t="s">
-        <v>166</v>
-      </c>
-      <c r="B28">
-        <v>13407</v>
-      </c>
-      <c r="C28">
-        <v>1994</v>
-      </c>
-      <c r="D28" t="s">
-        <v>179</v>
-      </c>
-      <c r="E28" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" t="s">
-        <v>109</v>
-      </c>
-      <c r="B29">
-        <v>13461</v>
-      </c>
-      <c r="C29">
-        <v>1926</v>
-      </c>
-      <c r="D29" t="s">
-        <v>179</v>
-      </c>
-      <c r="E29" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" t="s">
-        <v>138</v>
-      </c>
-      <c r="B30">
-        <v>13631</v>
-      </c>
-      <c r="C30">
-        <v>2001</v>
-      </c>
-      <c r="D30" t="s">
-        <v>176</v>
-      </c>
-      <c r="E30" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" t="s">
-        <v>130</v>
-      </c>
-      <c r="B31">
-        <v>13638</v>
-      </c>
-      <c r="C31">
-        <v>1963</v>
-      </c>
-      <c r="D31" t="s">
-        <v>179</v>
-      </c>
-      <c r="E31" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5">
-      <c r="A32" t="s">
-        <v>70</v>
-      </c>
-      <c r="B32">
-        <v>13762</v>
-      </c>
-      <c r="C32">
-        <v>1962</v>
-      </c>
-      <c r="D32" t="s">
-        <v>179</v>
-      </c>
-      <c r="E32" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
-      <c r="A33" t="s">
-        <v>98</v>
-      </c>
-      <c r="B33">
-        <v>13814</v>
-      </c>
-      <c r="C33">
-        <v>1928</v>
-      </c>
-      <c r="D33" t="s">
-        <v>179</v>
-      </c>
-      <c r="E33" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" t="s">
-        <v>96</v>
-      </c>
-      <c r="B34">
-        <v>14142</v>
-      </c>
-      <c r="C34">
-        <v>1912</v>
-      </c>
-      <c r="D34" t="s">
-        <v>179</v>
-      </c>
-      <c r="E34" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" t="s">
-        <v>126</v>
-      </c>
-      <c r="B35">
-        <v>14305</v>
-      </c>
-      <c r="C35">
-        <v>2047</v>
-      </c>
-      <c r="D35" t="s">
-        <v>179</v>
-      </c>
-      <c r="E35" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5">
-      <c r="A36" t="s">
-        <v>117</v>
-      </c>
-      <c r="B36">
-        <v>14444</v>
-      </c>
-      <c r="C36">
-        <v>2015</v>
-      </c>
-      <c r="D36" t="s">
-        <v>176</v>
-      </c>
-      <c r="E36" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5">
-      <c r="A37" t="s">
-        <v>119</v>
-      </c>
-      <c r="B37">
-        <v>14559</v>
-      </c>
-      <c r="C37">
-        <v>1994</v>
-      </c>
-      <c r="D37" t="s">
-        <v>176</v>
-      </c>
-      <c r="E37" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5">
-      <c r="A38" t="s">
-        <v>65</v>
-      </c>
-      <c r="B38">
-        <v>14665</v>
-      </c>
-      <c r="C38">
-        <v>2039</v>
-      </c>
-      <c r="D38" t="s">
-        <v>179</v>
-      </c>
-      <c r="E38" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5">
-      <c r="A39" t="s">
-        <v>82</v>
-      </c>
-      <c r="B39">
-        <v>14715</v>
-      </c>
-      <c r="C39">
-        <v>2002</v>
-      </c>
-      <c r="D39" t="s">
-        <v>179</v>
-      </c>
-      <c r="E39" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5">
-      <c r="A40" t="s">
-        <v>113</v>
-      </c>
-      <c r="B40">
-        <v>14763</v>
-      </c>
-      <c r="C40">
-        <v>2028</v>
-      </c>
-      <c r="D40" t="s">
-        <v>179</v>
-      </c>
-      <c r="E40" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5">
-      <c r="A41" t="s">
-        <v>168</v>
-      </c>
-      <c r="B41">
-        <v>14802</v>
-      </c>
-      <c r="C41">
-        <v>2038</v>
-      </c>
-      <c r="D41" t="s">
-        <v>179</v>
-      </c>
-      <c r="E41" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5">
-      <c r="A42" t="s">
-        <v>63</v>
-      </c>
-      <c r="B42">
-        <v>14861</v>
-      </c>
-      <c r="C42">
-        <v>2069</v>
-      </c>
-      <c r="D42" t="s">
-        <v>176</v>
-      </c>
-      <c r="E42" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5">
-      <c r="A43" t="s">
-        <v>136</v>
-      </c>
-      <c r="B43">
-        <v>14888</v>
-      </c>
-      <c r="C43">
-        <v>2080</v>
-      </c>
-      <c r="D43" t="s">
-        <v>176</v>
-      </c>
-      <c r="E43" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5">
-      <c r="A44" t="s">
-        <v>80</v>
-      </c>
-      <c r="B44">
-        <v>14920</v>
-      </c>
-      <c r="C44">
-        <v>2070</v>
-      </c>
-      <c r="D44" t="s">
-        <v>179</v>
-      </c>
-      <c r="E44" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5">
-      <c r="A45" t="s">
-        <v>72</v>
-      </c>
-      <c r="B45">
-        <v>15037</v>
-      </c>
-      <c r="C45">
-        <v>1966</v>
-      </c>
-      <c r="D45" t="s">
-        <v>179</v>
-      </c>
-      <c r="E45" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5">
-      <c r="A46" t="s">
-        <v>153</v>
-      </c>
-      <c r="B46">
-        <v>15218</v>
-      </c>
-      <c r="C46">
-        <v>1954</v>
-      </c>
-      <c r="D46" t="s">
-        <v>176</v>
-      </c>
-      <c r="E46" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5">
-      <c r="A47" t="s">
-        <v>149</v>
-      </c>
-      <c r="B47">
-        <v>15415</v>
-      </c>
-      <c r="C47">
-        <v>2061</v>
-      </c>
-      <c r="D47" t="s">
-        <v>176</v>
-      </c>
-      <c r="E47" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5">
-      <c r="A48" t="s">
-        <v>74</v>
-      </c>
-      <c r="B48">
-        <v>15641</v>
-      </c>
-      <c r="C48">
-        <v>2043</v>
-      </c>
-      <c r="D48" t="s">
-        <v>179</v>
-      </c>
-      <c r="E48" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5">
-      <c r="A49" t="s">
-        <v>68</v>
-      </c>
-      <c r="B49">
-        <v>16656</v>
-      </c>
-      <c r="C49">
-        <v>2070</v>
-      </c>
-      <c r="D49" t="s">
-        <v>179</v>
-      </c>
-      <c r="E49" t="s">
-        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3632,7 +3572,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -3648,793 +3588,750 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B2" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B3" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C3" t="s">
-        <v>186</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>187</v>
-      </c>
-      <c r="B2" t="s">
-        <v>188</v>
-      </c>
-      <c r="C2" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>190</v>
-      </c>
-      <c r="B3" t="s">
-        <v>191</v>
-      </c>
-      <c r="C3" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="B4" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="C4" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="B5" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="C5" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="B6" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="C6" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="B7" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="C7" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="B8" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="C8" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="B9" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="C9" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="B10" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C10" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="B11" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="C11" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="B12" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="C12" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="B13" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="C13" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="B14" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="C14" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="B15" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C15" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="B16" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="C16" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="B17" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="C17" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="B18" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="C18" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="B19" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="C19" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="B20" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="C20" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="B21" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="C21" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="B22" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="C22" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="B23" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="C23" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="B24" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="C24" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="B25" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="C25" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="B26" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="C26" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="B27" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="C27" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="B28" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="C28" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="B29" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="C29" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="B30" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="C30" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="B31" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="C31" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="B32" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="C32" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="B33" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="C33" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="B34" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="C34" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="B35" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="C35" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="B36" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="C36" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="B37" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="C37" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="B38" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="C38" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="B39" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="C39" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="B40" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="C40" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="B41" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="C41" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="B42" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="C42" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="B43" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="C43" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="B44" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="C44" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="B45" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="C45" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="B46" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="C46" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="B47" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="C47" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="B48" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="C48" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="B49" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="C49" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="B50" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="C50" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="B51" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="C51" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="B52" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="C52" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="B53" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="C53" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="B54" t="s">
-        <v>293</v>
+        <v>284</v>
       </c>
       <c r="C54" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="B55" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="C55" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="B56" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="C56" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="B57" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="C57" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="B58" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="C58" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="B59" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="C59" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>304</v>
+        <v>295</v>
       </c>
       <c r="B60" t="s">
-        <v>305</v>
+        <v>296</v>
       </c>
       <c r="C60" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>306</v>
+        <v>297</v>
       </c>
       <c r="B61" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="C61" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>308</v>
+        <v>299</v>
       </c>
       <c r="B62" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="C62" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>309</v>
+        <v>300</v>
       </c>
       <c r="B63" t="s">
-        <v>310</v>
+        <v>301</v>
       </c>
       <c r="C63" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>311</v>
+        <v>302</v>
       </c>
       <c r="B64" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="C64" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="B65" t="s">
-        <v>314</v>
+        <v>305</v>
       </c>
       <c r="C65" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="B66" t="s">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="C66" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="B67" t="s">
-        <v>318</v>
+        <v>309</v>
       </c>
       <c r="C67" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="B68" t="s">
-        <v>320</v>
+        <v>311</v>
       </c>
       <c r="C68" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="B69" t="s">
-        <v>322</v>
+        <v>313</v>
       </c>
       <c r="C69" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
trim the branch to what runs, so every folder here means something
</commit_message>
<xml_diff>
--- a/01_Processing/01_Precursors/c_data/precursors.xlsx
+++ b/01_Processing/01_Precursors/c_data/precursors.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="279">
   <si>
     <t>sheet</t>
   </si>
@@ -85,13 +85,13 @@
     <t>sample_id</t>
   </si>
   <si>
-    <t>One biopsy: subject_timepoint.</t>
+    <t>One biopsy: person and time point, e.g. S03_T1.</t>
   </si>
   <si>
     <t>injection</t>
   </si>
   <si>
-    <t>Injection suffix in the run name: empty for the first injection, r, rr, 4 or r for a re-injection.</t>
+    <t>Injection suffix in the run name: empty for the first injection; r, rr, _r or _4 for a re-injection.</t>
   </si>
   <si>
     <t>in_study</t>
@@ -133,7 +133,7 @@
     <t>group</t>
   </si>
   <si>
-    <t>Group the row belongs to: HR or LR, or C1 or C2 in a proteome grouping.</t>
+    <t>HR (higher responder) or LR (lower responder).</t>
   </si>
   <si>
     <t>timepoint</t>
@@ -556,228 +556,153 @@
     <t>deb1037f62a912aec543f05a585fe6d3</t>
   </si>
   <si>
-    <t>BiocGenerics</t>
-  </si>
-  <si>
-    <t>0.58.0</t>
+    <t>BiocManager</t>
+  </si>
+  <si>
+    <t>1.30.27</t>
+  </si>
+  <si>
+    <t>CRAN (R 4.6.0)</t>
+  </si>
+  <si>
+    <t>bit</t>
+  </si>
+  <si>
+    <t>4.6.0</t>
+  </si>
+  <si>
+    <t>bit64</t>
+  </si>
+  <si>
+    <t>4.8.0</t>
+  </si>
+  <si>
+    <t>cli</t>
+  </si>
+  <si>
+    <t>3.6.6</t>
+  </si>
+  <si>
+    <t>crayon</t>
+  </si>
+  <si>
+    <t>1.5.3</t>
+  </si>
+  <si>
+    <t>data.table</t>
+  </si>
+  <si>
+    <t>1.18.4</t>
+  </si>
+  <si>
+    <t>digest</t>
+  </si>
+  <si>
+    <t>0.6.39</t>
+  </si>
+  <si>
+    <t>dplyr</t>
+  </si>
+  <si>
+    <t>1.2.1</t>
+  </si>
+  <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
+  </si>
+  <si>
+    <t>farver</t>
+  </si>
+  <si>
+    <t>2.1.2</t>
+  </si>
+  <si>
+    <t>fastmap</t>
+  </si>
+  <si>
+    <t>1.2.0</t>
+  </si>
+  <si>
+    <t>generics</t>
+  </si>
+  <si>
+    <t>0.1.4</t>
+  </si>
+  <si>
+    <t>ggplot2</t>
+  </si>
+  <si>
+    <t>4.0.3</t>
+  </si>
+  <si>
+    <t>glue</t>
+  </si>
+  <si>
+    <t>1.8.1</t>
+  </si>
+  <si>
+    <t>gtable</t>
+  </si>
+  <si>
+    <t>0.3.6</t>
+  </si>
+  <si>
+    <t>here</t>
+  </si>
+  <si>
+    <t>1.0.2</t>
+  </si>
+  <si>
+    <t>hms</t>
+  </si>
+  <si>
+    <t>1.1.4</t>
+  </si>
+  <si>
+    <t>htmltools</t>
+  </si>
+  <si>
+    <t>0.5.9</t>
+  </si>
+  <si>
+    <t>htmlwidgets</t>
+  </si>
+  <si>
+    <t>1.6.4</t>
+  </si>
+  <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
+    <t>knitr</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
+    <t>labeling</t>
+  </si>
+  <si>
+    <t>0.4.3</t>
+  </si>
+  <si>
+    <t>lifecycle</t>
+  </si>
+  <si>
+    <t>limma</t>
+  </si>
+  <si>
+    <t>3.68.1</t>
   </si>
   <si>
     <t>Bioconductor 3.23 (R 4.6.0)</t>
   </si>
   <si>
-    <t>BiocManager</t>
-  </si>
-  <si>
-    <t>1.30.27</t>
-  </si>
-  <si>
-    <t>CRAN (R 4.6.0)</t>
-  </si>
-  <si>
-    <t>bit</t>
-  </si>
-  <si>
-    <t>4.6.0</t>
-  </si>
-  <si>
-    <t>bit64</t>
-  </si>
-  <si>
-    <t>4.8.0</t>
-  </si>
-  <si>
-    <t>circlize</t>
-  </si>
-  <si>
-    <t>0.4.18</t>
-  </si>
-  <si>
-    <t>cli</t>
-  </si>
-  <si>
-    <t>3.6.6</t>
-  </si>
-  <si>
-    <t>clue</t>
-  </si>
-  <si>
-    <t>0.3-68</t>
-  </si>
-  <si>
-    <t>cluster</t>
-  </si>
-  <si>
-    <t>2.1.8.2</t>
-  </si>
-  <si>
-    <t>codetools</t>
-  </si>
-  <si>
-    <t>0.2-20</t>
-  </si>
-  <si>
-    <t>colorspace</t>
-  </si>
-  <si>
-    <t>2.1-2</t>
-  </si>
-  <si>
-    <t>ComplexHeatmap</t>
-  </si>
-  <si>
-    <t>2.28.0</t>
-  </si>
-  <si>
-    <t>crayon</t>
-  </si>
-  <si>
-    <t>1.5.3</t>
-  </si>
-  <si>
-    <t>data.table</t>
-  </si>
-  <si>
-    <t>1.18.4</t>
-  </si>
-  <si>
-    <t>digest</t>
-  </si>
-  <si>
-    <t>0.6.39</t>
-  </si>
-  <si>
-    <t>doParallel</t>
-  </si>
-  <si>
-    <t>1.0.17</t>
-  </si>
-  <si>
-    <t>dplyr</t>
-  </si>
-  <si>
-    <t>1.2.1</t>
-  </si>
-  <si>
-    <t>evaluate</t>
-  </si>
-  <si>
-    <t>1.0.5</t>
-  </si>
-  <si>
-    <t>farver</t>
-  </si>
-  <si>
-    <t>2.1.2</t>
-  </si>
-  <si>
-    <t>fastmap</t>
-  </si>
-  <si>
-    <t>1.2.0</t>
-  </si>
-  <si>
-    <t>foreach</t>
-  </si>
-  <si>
-    <t>1.5.2</t>
-  </si>
-  <si>
-    <t>generics</t>
-  </si>
-  <si>
-    <t>0.1.4</t>
-  </si>
-  <si>
-    <t>GetoptLong</t>
-  </si>
-  <si>
-    <t>1.1.1</t>
-  </si>
-  <si>
-    <t>ggplot2</t>
-  </si>
-  <si>
-    <t>4.0.3</t>
-  </si>
-  <si>
-    <t>GlobalOptions</t>
-  </si>
-  <si>
-    <t>glue</t>
-  </si>
-  <si>
-    <t>1.8.1</t>
-  </si>
-  <si>
-    <t>gtable</t>
-  </si>
-  <si>
-    <t>0.3.6</t>
-  </si>
-  <si>
-    <t>here</t>
-  </si>
-  <si>
-    <t>1.0.2</t>
-  </si>
-  <si>
-    <t>hms</t>
-  </si>
-  <si>
-    <t>1.1.4</t>
-  </si>
-  <si>
-    <t>htmltools</t>
-  </si>
-  <si>
-    <t>0.5.9</t>
-  </si>
-  <si>
-    <t>htmlwidgets</t>
-  </si>
-  <si>
-    <t>1.6.4</t>
-  </si>
-  <si>
-    <t>IRanges</t>
-  </si>
-  <si>
-    <t>2.46.0</t>
-  </si>
-  <si>
-    <t>iterators</t>
-  </si>
-  <si>
-    <t>1.0.14</t>
-  </si>
-  <si>
-    <t>jsonlite</t>
-  </si>
-  <si>
-    <t>2.0.0</t>
-  </si>
-  <si>
-    <t>knitr</t>
-  </si>
-  <si>
-    <t>1.51</t>
-  </si>
-  <si>
-    <t>labeling</t>
-  </si>
-  <si>
-    <t>0.4.3</t>
-  </si>
-  <si>
-    <t>lifecycle</t>
-  </si>
-  <si>
-    <t>limma</t>
-  </si>
-  <si>
-    <t>3.68.1</t>
-  </si>
-  <si>
     <t>limpa</t>
   </si>
   <si>
@@ -790,12 +715,6 @@
     <t>2.0.5</t>
   </si>
   <si>
-    <t>matrixStats</t>
-  </si>
-  <si>
-    <t>1.5.0</t>
-  </si>
-  <si>
     <t>nanoparquet</t>
   </si>
   <si>
@@ -823,12 +742,6 @@
     <t>2.0.3</t>
   </si>
   <si>
-    <t>png</t>
-  </si>
-  <si>
-    <t>0.1-9</t>
-  </si>
-  <si>
     <t>R6</t>
   </si>
   <si>
@@ -853,12 +766,6 @@
     <t>1.2.3</t>
   </si>
   <si>
-    <t>rjson</t>
-  </si>
-  <si>
-    <t>0.2.23</t>
-  </si>
-  <si>
     <t>rlang</t>
   </si>
   <si>
@@ -877,12 +784,6 @@
     <t>2.1.1</t>
   </si>
   <si>
-    <t>S4Vectors</t>
-  </si>
-  <si>
-    <t>0.50.0</t>
-  </si>
-  <si>
     <t>S7</t>
   </si>
   <si>
@@ -899,12 +800,6 @@
   </si>
   <si>
     <t>1.2.4</t>
-  </si>
-  <si>
-    <t>shape</t>
-  </si>
-  <si>
-    <t>1.4.6.1</t>
   </si>
   <si>
     <t>statmod</t>
@@ -3572,7 +3467,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -3605,103 +3500,103 @@
         <v>182</v>
       </c>
       <c r="C3" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B4" t="s">
         <v>184</v>
       </c>
-      <c r="B4" t="s">
-        <v>185</v>
-      </c>
       <c r="C4" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B5" t="s">
         <v>186</v>
       </c>
-      <c r="B5" t="s">
-        <v>187</v>
-      </c>
       <c r="C5" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
+        <v>187</v>
+      </c>
+      <c r="B6" t="s">
         <v>188</v>
       </c>
-      <c r="B6" t="s">
-        <v>189</v>
-      </c>
       <c r="C6" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
+        <v>189</v>
+      </c>
+      <c r="B7" t="s">
         <v>190</v>
       </c>
-      <c r="B7" t="s">
-        <v>191</v>
-      </c>
       <c r="C7" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
+        <v>191</v>
+      </c>
+      <c r="B8" t="s">
         <v>192</v>
       </c>
-      <c r="B8" t="s">
-        <v>193</v>
-      </c>
       <c r="C8" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
+        <v>193</v>
+      </c>
+      <c r="B9" t="s">
         <v>194</v>
       </c>
-      <c r="B9" t="s">
-        <v>195</v>
-      </c>
       <c r="C9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
+        <v>195</v>
+      </c>
+      <c r="B10" t="s">
         <v>196</v>
       </c>
-      <c r="B10" t="s">
-        <v>197</v>
-      </c>
       <c r="C10" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
+        <v>197</v>
+      </c>
+      <c r="B11" t="s">
         <v>198</v>
       </c>
-      <c r="B11" t="s">
-        <v>199</v>
-      </c>
       <c r="C11" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
+        <v>199</v>
+      </c>
+      <c r="B12" t="s">
         <v>200</v>
-      </c>
-      <c r="B12" t="s">
-        <v>201</v>
       </c>
       <c r="C12" t="s">
         <v>180</v>
@@ -3709,145 +3604,145 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
+        <v>201</v>
+      </c>
+      <c r="B13" t="s">
         <v>202</v>
       </c>
-      <c r="B13" t="s">
-        <v>203</v>
-      </c>
       <c r="C13" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
+        <v>203</v>
+      </c>
+      <c r="B14" t="s">
         <v>204</v>
       </c>
-      <c r="B14" t="s">
-        <v>205</v>
-      </c>
       <c r="C14" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
+        <v>205</v>
+      </c>
+      <c r="B15" t="s">
         <v>206</v>
       </c>
-      <c r="B15" t="s">
-        <v>207</v>
-      </c>
       <c r="C15" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
+        <v>207</v>
+      </c>
+      <c r="B16" t="s">
         <v>208</v>
       </c>
-      <c r="B16" t="s">
-        <v>209</v>
-      </c>
       <c r="C16" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
+        <v>209</v>
+      </c>
+      <c r="B17" t="s">
         <v>210</v>
       </c>
-      <c r="B17" t="s">
-        <v>211</v>
-      </c>
       <c r="C17" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
+        <v>211</v>
+      </c>
+      <c r="B18" t="s">
         <v>212</v>
       </c>
-      <c r="B18" t="s">
-        <v>213</v>
-      </c>
       <c r="C18" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
+        <v>213</v>
+      </c>
+      <c r="B19" t="s">
         <v>214</v>
       </c>
-      <c r="B19" t="s">
-        <v>215</v>
-      </c>
       <c r="C19" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
+        <v>215</v>
+      </c>
+      <c r="B20" t="s">
         <v>216</v>
       </c>
-      <c r="B20" t="s">
-        <v>217</v>
-      </c>
       <c r="C20" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
+        <v>217</v>
+      </c>
+      <c r="B21" t="s">
         <v>218</v>
       </c>
-      <c r="B21" t="s">
-        <v>219</v>
-      </c>
       <c r="C21" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
+        <v>219</v>
+      </c>
+      <c r="B22" t="s">
         <v>220</v>
       </c>
-      <c r="B22" t="s">
-        <v>221</v>
-      </c>
       <c r="C22" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
+        <v>221</v>
+      </c>
+      <c r="B23" t="s">
         <v>222</v>
       </c>
-      <c r="B23" t="s">
-        <v>223</v>
-      </c>
       <c r="C23" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B24" t="s">
-        <v>225</v>
+        <v>196</v>
       </c>
       <c r="C24" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>224</v>
+      </c>
+      <c r="B25" t="s">
+        <v>225</v>
+      </c>
+      <c r="C25" t="s">
         <v>226</v>
-      </c>
-      <c r="B25" t="s">
-        <v>221</v>
-      </c>
-      <c r="C25" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -3858,7 +3753,7 @@
         <v>228</v>
       </c>
       <c r="C26" t="s">
-        <v>183</v>
+        <v>226</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -3869,7 +3764,7 @@
         <v>230</v>
       </c>
       <c r="C27" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -3880,48 +3775,48 @@
         <v>232</v>
       </c>
       <c r="C28" t="s">
-        <v>183</v>
+        <v>233</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B29" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C29" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B30" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C30" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B31" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C31" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B32" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C32" t="s">
         <v>180</v>
@@ -3929,65 +3824,65 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B33" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C33" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B34" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C34" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B35" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C35" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B36" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C36" t="s">
-        <v>183</v>
+        <v>233</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B37" t="s">
-        <v>213</v>
+        <v>251</v>
       </c>
       <c r="C37" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B38" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C38" t="s">
         <v>180</v>
@@ -3995,10 +3890,10 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B39" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C39" t="s">
         <v>180</v>
@@ -4006,57 +3901,57 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B40" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C40" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B41" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C41" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B42" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C42" t="s">
-        <v>260</v>
+        <v>180</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B43" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C43" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B44" t="s">
-        <v>264</v>
+        <v>194</v>
       </c>
       <c r="C44" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -4067,7 +3962,7 @@
         <v>266</v>
       </c>
       <c r="C45" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -4078,7 +3973,7 @@
         <v>268</v>
       </c>
       <c r="C46" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -4089,7 +3984,7 @@
         <v>270</v>
       </c>
       <c r="C47" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -4100,7 +3995,7 @@
         <v>272</v>
       </c>
       <c r="C48" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -4111,7 +4006,7 @@
         <v>274</v>
       </c>
       <c r="C49" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -4122,7 +4017,7 @@
         <v>276</v>
       </c>
       <c r="C50" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -4133,205 +4028,7 @@
         <v>278</v>
       </c>
       <c r="C51" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="A52" t="s">
-        <v>279</v>
-      </c>
-      <c r="B52" t="s">
-        <v>280</v>
-      </c>
-      <c r="C52" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53" t="s">
-        <v>281</v>
-      </c>
-      <c r="B53" t="s">
-        <v>282</v>
-      </c>
-      <c r="C53" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3">
-      <c r="A54" t="s">
-        <v>283</v>
-      </c>
-      <c r="B54" t="s">
-        <v>284</v>
-      </c>
-      <c r="C54" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="A55" t="s">
-        <v>285</v>
-      </c>
-      <c r="B55" t="s">
-        <v>286</v>
-      </c>
-      <c r="C55" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3">
-      <c r="A56" t="s">
-        <v>287</v>
-      </c>
-      <c r="B56" t="s">
-        <v>288</v>
-      </c>
-      <c r="C56" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3">
-      <c r="A57" t="s">
-        <v>289</v>
-      </c>
-      <c r="B57" t="s">
-        <v>290</v>
-      </c>
-      <c r="C57" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3">
-      <c r="A58" t="s">
-        <v>291</v>
-      </c>
-      <c r="B58" t="s">
-        <v>292</v>
-      </c>
-      <c r="C58" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3">
-      <c r="A59" t="s">
-        <v>293</v>
-      </c>
-      <c r="B59" t="s">
-        <v>294</v>
-      </c>
-      <c r="C59" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3">
-      <c r="A60" t="s">
-        <v>295</v>
-      </c>
-      <c r="B60" t="s">
-        <v>296</v>
-      </c>
-      <c r="C60" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3">
-      <c r="A61" t="s">
-        <v>297</v>
-      </c>
-      <c r="B61" t="s">
-        <v>298</v>
-      </c>
-      <c r="C61" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3">
-      <c r="A62" t="s">
-        <v>299</v>
-      </c>
-      <c r="B62" t="s">
-        <v>211</v>
-      </c>
-      <c r="C62" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3">
-      <c r="A63" t="s">
-        <v>300</v>
-      </c>
-      <c r="B63" t="s">
-        <v>301</v>
-      </c>
-      <c r="C63" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3">
-      <c r="A64" t="s">
-        <v>302</v>
-      </c>
-      <c r="B64" t="s">
-        <v>303</v>
-      </c>
-      <c r="C64" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3">
-      <c r="A65" t="s">
-        <v>304</v>
-      </c>
-      <c r="B65" t="s">
-        <v>305</v>
-      </c>
-      <c r="C65" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3">
-      <c r="A66" t="s">
-        <v>306</v>
-      </c>
-      <c r="B66" t="s">
-        <v>307</v>
-      </c>
-      <c r="C66" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3">
-      <c r="A67" t="s">
-        <v>308</v>
-      </c>
-      <c r="B67" t="s">
-        <v>309</v>
-      </c>
-      <c r="C67" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3">
-      <c r="A68" t="s">
-        <v>310</v>
-      </c>
-      <c r="B68" t="s">
-        <v>311</v>
-      </c>
-      <c r="C68" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3">
-      <c r="A69" t="s">
-        <v>312</v>
-      </c>
-      <c r="B69" t="s">
-        <v>313</v>
-      </c>
-      <c r="C69" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>